<commit_message>
feat(data): generate and publish all 10 enterprise leads and proposals
</commit_message>
<xml_diff>
--- a/ai/output/sample_leads_proposals/Lead_01_Retail_Omnichannel.xlsx
+++ b/ai/output/sample_leads_proposals/Lead_01_Retail_Omnichannel.xlsx
@@ -503,7 +503,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>From: NovaRetail Holdings Pty Ltd     |     Date sent: 5 October 2026     |     Contact: Marcus Vance</t>
+          <t>From: NovaRetail Holdings Pty Ltd     |     Date sent: 05 October 2026     |     Contact: Marcus Vance – VP of Digital &amp; Omnichannel Operations (marcus.vance@novaretail.example | +61 2 9000 1234)</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
       </c>
       <c r="B4" s="4" t="n"/>
     </row>
-    <row r="5" ht="22" customHeight="1">
+    <row r="5" ht="24" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Company</t>
@@ -527,7 +527,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6" ht="32" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>What we do</t>
@@ -535,11 +535,11 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>We are a fashion and lifestyle apparel retailer with both physical retail stores and a fast-growing digital direct-to-consumer presence.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="55" customHeight="1">
+          <t>We are a fashion and lifestyle apparel retailer with physical retail stores and an online brand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="64" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Our footprint</t>
@@ -549,11 +549,11 @@
         <is>
           <t>- 120 physical retail stores across Australia, New Zealand, and Singapore (75 in Australia, 25 in NZ, 20 in SG)
 - 3 central distribution warehouses (Sydney, Melbourne, and Singapore)
-- Flagship online store on Shopify Plus (we average around 8,000 orders a day, peaking up to 35,000 orders a day during peak sale periods like Black Friday)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
+- Flagship online store on Shopify Plus (averages ~8,000 orders/day, up to 35,000 on peak sale days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="54" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -575,7 +575,7 @@
       </c>
       <c r="B9" s="4" t="n"/>
     </row>
-    <row r="10" ht="65" customHeight="1">
+    <row r="10" ht="80" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Current setup</t>
@@ -587,7 +587,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="155" customHeight="1">
+    <row r="11" ht="220" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>What isn't working for us (Our biggest headaches)</t>
@@ -595,7 +595,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>- Overselling and cancellations: Because our stores only upload stock twice a day, customers often buy items online that were already purchased off the rack in a store an hour earlier. During last year's Click Frenzy, we had to cancel 420 orders and pay out over $85,000 in apology vouchers to furious shoppers.
+          <t>- Overselling and cancellations: Because our stores only upload stock twice a day, customers often buy items online that were already purchased off the rack in a store an hour earlier. During last Click Frenzy, we had to cancel 420 orders and pay out over $85,000 in apology vouchers to furious shoppers.
 - Expensive and slow shipping: Right now, every single online order gets routed to our central warehouses in Sydney or Melbourne, even when a customer lives 10 minutes away from our Bondi or Chadstone store that has 5 units of the exact dress sitting on the shelf. This costs us around $14 per parcel in shipping and takes 3 to 4 days.
 - Warehouse picking errors: In our distribution centers, pickers spend half their shift walking back and forth with paper lists. They manually check items off with pens, and about 2.8% of parcels end up being shipped with the wrong size or wrong color.
 - Messy Click &amp; Collect: When a customer orders for store pickup, our store staff simply get an email. When the customer shows up, staff have to hunt through unorganized boxes in the back room while the customer waits 20 minutes at the counter.
@@ -611,7 +611,7 @@
       </c>
       <c r="B12" s="4" t="n"/>
     </row>
-    <row r="13" ht="55" customHeight="1">
+    <row r="13" ht="64" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>In short</t>
@@ -623,7 +623,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="90" customHeight="1">
+    <row r="14" ht="176" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Key things we need it to do</t>
@@ -647,7 +647,7 @@
       </c>
       <c r="B15" s="4" t="n"/>
     </row>
-    <row r="16" ht="75" customHeight="1">
+    <row r="16" ht="90" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Integrations</t>
@@ -671,7 +671,7 @@
       </c>
       <c r="B17" s="4" t="n"/>
     </row>
-    <row r="18" ht="75" customHeight="1">
+    <row r="18" ht="80" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Expectations</t>

</xml_diff>